<commit_message>
Enhance CT Imaging and Analysis Functionality
- Added README.md file for project documentation.
- Updated onClickCallback.m to implement a new colormap (turbo) for better visualization of concentration images.
- Modified main_CTimaging.m to comment out the imaging movie generation section for improved code clarity and maintainability.
- Refactored main_CTplots.m to streamline the plotting process and improve the organization of the code, including the removal of unnecessary sections related to movie generation.
- Enhanced main_CTpreproc.m to include the calculation of 2D velocity fields from iso-concentration contours and the displacement of contours between frames, improving the analysis of concentration dynamics.
- Updated inputCTExpConfig.xlsx to reflect changes in input parameters and configurations.
</commit_message>
<xml_diff>
--- a/inputCTExpConfig.xlsx
+++ b/inputCTExpConfig.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CT-Dispersion-Exps-Analog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA3E46C5-E462-41C5-A5DC-54D45AF11DB4}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{594BD307-6CB4-4FE8-87B4-12734FC3CFD0}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25575" yWindow="2265" windowWidth="23010" windowHeight="12030" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="All" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="17">
   <si>
     <t>inputFileName</t>
   </si>
@@ -54,10 +55,28 @@
     <t>importPath</t>
   </si>
   <si>
-    <t>input/input_exp_He-Xe-T20_test.xlsx</t>
-  </si>
-  <si>
     <t>results/CT_He-Xe-T20-P725-V-Q5/</t>
+  </si>
+  <si>
+    <t>input/input_exp_He-Xe-T20_P900_Q1.xlsx</t>
+  </si>
+  <si>
+    <t>results/CT_He-Xe-T20-P900-V-Q1/</t>
+  </si>
+  <si>
+    <t>input/input_exp_He-Xe-T20_P900_Q5.xlsx</t>
+  </si>
+  <si>
+    <t>results/CT_He-Xe-T20-P900-V-Q5/</t>
+  </si>
+  <si>
+    <t>input/input_exp_He-Xe-T20_P725_Q1.xlsx</t>
+  </si>
+  <si>
+    <t>results/CT_He-Xe-T20-P725-V-Q1/</t>
+  </si>
+  <si>
+    <t>input/input_exp_He-Xe-T20_P725_Q5.xlsx</t>
   </si>
 </sst>
 </file>
@@ -408,10 +427,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
@@ -420,6 +442,116 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FFD9648-A5F1-4DDE-8340-F889A16E0746}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>